<commit_message>
Update reports 2026-10-21 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-21.xlsx
+++ b/gex_pivot_levels_2026-10-21.xlsx
@@ -532,7 +532,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>7716.68</v>
+        <v>7716.18</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>7650</v>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$9.59M</t>
+          <t>-$10.43M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$11.69M</t>
+          <t>+$12.70M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -565,7 +565,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>7726.68</v>
+        <v>7726.18</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>7660</v>
@@ -577,12 +577,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$1.42M</t>
+          <t>-$1.57M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$6.85M</t>
+          <t>+$7.58M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -597,149 +597,157 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>7736.68</v>
-      </c>
-      <c r="B4" s="5" t="n">
+      <c r="A4" s="2" t="n">
+        <v>7736.18</v>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>7670</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>-$10.51M</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>+$12.70M</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-$11.74M</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>+$14.19M</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>7748.66</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>766</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>-$12.88M</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>+$19.50M</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A5" s="5" t="n">
+        <v>7741.18</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7675</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-$5.31M</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>+$8.92M</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>7766.68</v>
+        <v>7748.16</v>
       </c>
       <c r="B6" s="2" t="n">
+        <v>766</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-$12.88M</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>+$19.50M</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>7766.18</v>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>7700</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>-$19.09M</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>+$37.14M</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-$23.41M</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$45.54M</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>7776.68</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>7710</v>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>-$884.55K</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>+$17.73M</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>7778.75</v>
+        <v>7776.18</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>769</v>
+        <v>7710</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>+$6.06M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>-$3.58M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$33.87M</t>
+          <t>+$19.76M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -751,189 +759,181 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>7788.78</v>
+        <v>7778.25</v>
       </c>
       <c r="B9" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>+$6.06M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$33.87M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>7788.28</v>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>770</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>+$11.64M</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>+$29.49M</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>7791.68</v>
-      </c>
-      <c r="B10" s="2" t="n">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>7791.18</v>
+      </c>
+      <c r="B11" s="2" t="n">
         <v>7725</v>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>+$20.16M</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>+$40.40M</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>7796.68</v>
-      </c>
-      <c r="B11" s="5" t="n">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>+$9.34M</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>+$35.81M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>7796.18</v>
+      </c>
+      <c r="B12" s="5" t="n">
         <v>7730</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>+$6.79M</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>+$14.79M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>+$2.66M</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>+$13.21M</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>7806.68</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>7740</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>+$16.94M</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>+$22.11M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>7808.83</v>
+        <v>7806.18</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>772</v>
+        <v>7740</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$3.58M</t>
+          <t>+$11.36M</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>+$17.47M</t>
+          <t>+$18.26M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>7811.68</v>
+        <v>7808.33</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7745</v>
+        <v>772</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$8.51M</t>
+          <t>+$3.58M</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>+$12.72M</t>
+          <t>+$17.47M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -949,7 +949,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>7816.68</v>
+        <v>7816.18</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>7750</v>
@@ -961,12 +961,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>+$27.95M</t>
+          <t>+$17.32M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$43.53M</t>
+          <t>+$37.76M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -982,7 +982,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>7818.86</v>
+        <v>7818.36</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>773</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>7821.68</v>
+        <v>7821.18</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>7755</v>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$12.78M</t>
+          <t>+$9.30M</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$15.24M</t>
+          <t>+$12.47M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1048,7 +1048,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>7826.68</v>
+        <v>7826.18</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>7760</v>
@@ -1060,12 +1060,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>+$17.08M</t>
+          <t>+$11.67M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$24.61M</t>
+          <t>+$21.25M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1077,7 +1077,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>7828.89</v>
+        <v>7828.39</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>774</v>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>7841.68</v>
+        <v>7841.18</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>7775</v>
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$24.06M</t>
+          <t>+$18.32M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$31.91M</t>
+          <t>+$27.11M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1143,7 +1143,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>7848.95</v>
+        <v>7848.45</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>776</v>
@@ -1176,7 +1176,7 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>7866.68</v>
+        <v>7866.18</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>7800</v>
@@ -1188,12 +1188,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$5.59M</t>
+          <t>+$5.21M</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>+$15.28M</t>
+          <t>+$11.49M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1267,7 +1267,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>29245.26</v>
+        <v>29195.26</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>700</v>
@@ -1300,7 +1300,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>29286.36</v>
+        <v>29236.36</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>701</v>
@@ -1333,7 +1333,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>29450.73</v>
+        <v>29400.73</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>705</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>29491.83</v>
+        <v>29441.83</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>706</v>
@@ -1399,7 +1399,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>29656.2</v>
+        <v>29606.2</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>710</v>
@@ -1432,7 +1432,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>29759.47</v>
+        <v>29709.47</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>29280</v>
@@ -1461,7 +1461,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>29779.47</v>
+        <v>29729.47</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>29300</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>29779.48</v>
+        <v>29729.48</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>713</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>29799.47</v>
+        <v>29749.47</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>29320</v>
@@ -1556,7 +1556,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>29829.47</v>
+        <v>29779.47</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>29350</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>29854.47</v>
+        <v>29804.47</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>29375</v>
@@ -1622,7 +1622,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>29861.67</v>
+        <v>29811.67</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>715</v>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>29879.47</v>
+        <v>29829.47</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>29400</v>
@@ -1688,7 +1688,7 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>29899.47</v>
+        <v>29849.47</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>29420</v>
@@ -1721,7 +1721,7 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>29902.77</v>
+        <v>29852.77</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>716</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>29929.47</v>
+        <v>29879.47</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>29450</v>
@@ -1787,7 +1787,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>29939.47</v>
+        <v>29889.47</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>29460</v>
@@ -1820,7 +1820,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>29943.86</v>
+        <v>29893.86</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>717</v>
@@ -1853,7 +1853,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>29959.47</v>
+        <v>29909.47</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>29480</v>
@@ -1886,7 +1886,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>29969.47</v>
+        <v>29919.47</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>29490</v>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>29979.47</v>
+        <v>29929.47</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>29500</v>
@@ -1952,7 +1952,7 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>29984.95</v>
+        <v>29934.95</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>718</v>
@@ -1981,7 +1981,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>29999.47</v>
+        <v>29949.47</v>
       </c>
       <c r="B24" s="5" t="n">
         <v>29520</v>
@@ -2010,7 +2010,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>30009.47</v>
+        <v>29959.47</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>29530</v>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
-        <v>30029.47</v>
+        <v>29979.47</v>
       </c>
       <c r="B26" s="5" t="n">
         <v>29550</v>
@@ -2072,7 +2072,7 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>30049.47</v>
+        <v>29999.47</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>29570</v>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>30059.47</v>
+        <v>30009.47</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>29580</v>
@@ -2138,7 +2138,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>30067.14</v>
+        <v>30017.14</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>720</v>
@@ -2171,7 +2171,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>30079.47</v>
+        <v>30029.47</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>29600</v>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>30108.24</v>
+        <v>30058.24</v>
       </c>
       <c r="B31" s="5" t="n">
         <v>721</v>
@@ -2237,7 +2237,7 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
-        <v>30129.47</v>
+        <v>30079.47</v>
       </c>
       <c r="B32" s="5" t="n">
         <v>29650</v>
@@ -2266,7 +2266,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>30272.61</v>
+        <v>30222.61</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>725</v>
@@ -2299,7 +2299,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
-        <v>30436.99</v>
+        <v>30386.99</v>
       </c>
       <c r="B34" s="5" t="n">
         <v>729</v>
@@ -2332,7 +2332,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>30478.08</v>
+        <v>30428.08</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>730</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>92.63</v>
+        <v>92.69</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>150</v>
@@ -2617,7 +2617,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>95.72</v>
+        <v>95.78</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>155</v>
@@ -2650,7 +2650,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>96.33</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>156</v>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>98.8</v>
+        <v>98.87</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>160</v>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>101.89</v>
+        <v>101.96</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>165</v>
@@ -2749,7 +2749,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>104.36</v>
+        <v>104.43</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>169</v>
@@ -2782,7 +2782,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>104.98</v>
+        <v>105.05</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>170</v>
@@ -3480,24 +3480,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7816.68</v>
+        <v>7766.18</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7750</v>
+        <v>7700</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>+$27.95M</t>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>-$23.41M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$43.53M</t>
+          <t>+$45.54M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3518,10 +3518,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>7791.68</v>
+        <v>7816.18</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7725</v>
+        <v>7750</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -3530,12 +3530,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$20.16M</t>
+          <t>+$17.32M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$40.40M</t>
+          <t>+$37.76M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3556,24 +3556,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7766.68</v>
+        <v>7791.18</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7700</v>
+        <v>7725</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>-$19.09M</t>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>+$9.34M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$37.14M</t>
+          <t>+$35.81M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7778.75</v>
+        <v>7778.25</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>769</v>
@@ -3628,108 +3628,108 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>7841.68</v>
+        <v>7818.36</v>
       </c>
       <c r="C8" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>+$8.15M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>+$31.72M</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7788.28</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>+$11.64M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>+$29.49M</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>7841.18</v>
+      </c>
+      <c r="C10" s="2" t="n">
         <v>7775</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>+$24.06M</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>+$31.91M</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>7818.86</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>773</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>+$8.15M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>+$31.72M</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>7788.78</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>770</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>+$11.64M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>+$29.49M</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>+$18.32M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>+$27.11M</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3742,7 +3742,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>30067.14</v>
+        <v>30017.14</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>720</v>
@@ -3780,7 +3780,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7828.89</v>
+        <v>7828.39</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>774</v>
@@ -3818,7 +3818,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7826.68</v>
+        <v>7826.18</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>7760</v>
@@ -3830,12 +3830,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>+$17.08M</t>
+          <t>+$11.67M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>+$24.61M</t>
+          <t>+$21.25M</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -3846,42 +3846,38 @@
       <c r="H13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>7806.68</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>7740</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="n">
+        <v>7776.18</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>7710</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$16.94M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$22.11M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-$3.58M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$19.76M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3890,7 +3886,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7748.66</v>
+        <v>7748.16</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>766</v>
@@ -3928,24 +3924,24 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>7776.68</v>
+        <v>7806.18</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>7710</v>
+        <v>7740</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-$884.55K</t>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>+$17.73M</t>
+          <t>+$18.26M</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -3962,7 +3958,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>7808.83</v>
+        <v>7808.33</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>772</v>
@@ -3994,38 +3990,42 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>7866.68</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="B18" s="2" t="n">
+        <v>7736.18</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>7670</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>+$5.59M</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>+$15.28M</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>-$11.74M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>+$14.19M</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -4034,10 +4034,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>7821.68</v>
+        <v>7796.18</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>7755</v>
+        <v>7730</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -4046,12 +4046,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>+$12.78M</t>
+          <t>+$2.66M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$15.24M</t>
+          <t>+$13.21M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -4066,38 +4066,38 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>7796.68</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>7730</v>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>+$6.79M</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>+$14.79M</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>29606.2</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>710</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$8.02M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>+$12.81M</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4106,28 +4106,28 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>29656.2</v>
+        <v>7716.18</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>710</v>
+        <v>7650</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>-$8.02M</t>
+          <t>-$10.43M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>+$12.81M</t>
+          <t>+$12.70M</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -4148,10 +4148,10 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7811.68</v>
+        <v>7821.18</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>7745</v>
+        <v>7755</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -4160,12 +4160,12 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>+$8.51M</t>
+          <t>+$9.30M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$12.72M</t>
+          <t>+$12.47M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -4186,180 +4186,180 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7736.68</v>
+        <v>7848.45</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>7670</v>
+        <v>776</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-$10.51M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>+$6.50M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>+$12.70M</t>
+          <t>+$12.00M</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2776.56</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>276</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>+$4.91M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>+$11.66M</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
-        <v>7848.95</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>776</v>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>+$6.50M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>+$12.00M</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7716.68</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="B25" s="5" t="n">
+        <v>7866.18</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-$9.59M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$11.69M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$5.21M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$11.49M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2776.56</v>
+        <v>29934.95</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>276</v>
+        <v>718</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$4.91M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-$821.63K</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$11.66M</t>
+          <t>+$9.99M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>29984.95</v>
+        <v>7741.18</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>718</v>
+        <v>7675</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>-$821.63K</t>
+          <t>-$5.31M</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>+$9.99M</t>
+          <t>+$8.92M</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -4368,7 +4368,7 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>30272.61</v>
+        <v>30222.61</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>725</v>
@@ -4406,7 +4406,7 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>29861.67</v>
+        <v>29811.67</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>715</v>
@@ -4444,7 +4444,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>7726.68</v>
+        <v>7726.18</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>7660</v>
@@ -4456,12 +4456,12 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>-$1.42M</t>
+          <t>-$1.57M</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>+$6.85M</t>
+          <t>+$7.58M</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -4482,7 +4482,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>29943.86</v>
+        <v>29893.86</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>717</v>
@@ -4520,7 +4520,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>30478.08</v>
+        <v>30428.08</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>730</v>
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>30108.24</v>
+        <v>30058.24</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>721</v>
@@ -4596,7 +4596,7 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>29245.26</v>
+        <v>29195.26</v>
       </c>
       <c r="C34" s="2" t="n">
         <v>700</v>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>101.89</v>
+        <v>101.96</v>
       </c>
       <c r="C35" s="2" t="n">
         <v>165</v>
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>29450.73</v>
+        <v>29400.73</v>
       </c>
       <c r="C36" s="2" t="n">
         <v>705</v>
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>29902.77</v>
+        <v>29852.77</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>716</v>
@@ -4748,7 +4748,7 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>29779.48</v>
+        <v>29729.48</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>713</v>
@@ -4786,7 +4786,7 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>98.8</v>
+        <v>98.87</v>
       </c>
       <c r="C39" s="2" t="n">
         <v>160</v>
@@ -4824,7 +4824,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>30436.99</v>
+        <v>30386.99</v>
       </c>
       <c r="C40" s="5" t="n">
         <v>729</v>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>104.98</v>
+        <v>105.05</v>
       </c>
       <c r="C41" s="2" t="n">
         <v>170</v>
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>95.72</v>
+        <v>95.78</v>
       </c>
       <c r="C43" s="2" t="n">
         <v>155</v>
@@ -5120,7 +5120,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>96.33</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="C48" s="5" t="n">
         <v>156</v>
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>29491.83</v>
+        <v>29441.83</v>
       </c>
       <c r="C50" s="5" t="n">
         <v>706</v>
@@ -5272,7 +5272,7 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>92.63</v>
+        <v>92.69</v>
       </c>
       <c r="C52" s="5" t="n">
         <v>150</v>
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>29286.36</v>
+        <v>29236.36</v>
       </c>
       <c r="C57" s="5" t="n">
         <v>701</v>
@@ -5496,7 +5496,7 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>30009.47</v>
+        <v>29959.47</v>
       </c>
       <c r="C58" s="2" t="n">
         <v>29530</v>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>29979.47</v>
+        <v>29929.47</v>
       </c>
       <c r="C59" s="2" t="n">
         <v>29500</v>
@@ -5610,7 +5610,7 @@
         </is>
       </c>
       <c r="B61" s="5" t="n">
-        <v>29999.47</v>
+        <v>29949.47</v>
       </c>
       <c r="C61" s="5" t="n">
         <v>29520</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>29959.47</v>
+        <v>29909.47</v>
       </c>
       <c r="C62" s="2" t="n">
         <v>29480</v>
@@ -5682,7 +5682,7 @@
         </is>
       </c>
       <c r="B63" s="5" t="n">
-        <v>104.36</v>
+        <v>104.43</v>
       </c>
       <c r="C63" s="5" t="n">
         <v>169</v>
@@ -5720,7 +5720,7 @@
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>30029.47</v>
+        <v>29979.47</v>
       </c>
       <c r="C64" s="5" t="n">
         <v>29550</v>
@@ -5792,7 +5792,7 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>30079.47</v>
+        <v>30029.47</v>
       </c>
       <c r="C66" s="2" t="n">
         <v>29600</v>
@@ -5830,7 +5830,7 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>29879.47</v>
+        <v>29829.47</v>
       </c>
       <c r="C67" s="2" t="n">
         <v>29400</v>
@@ -5868,7 +5868,7 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>30059.47</v>
+        <v>30009.47</v>
       </c>
       <c r="C68" s="2" t="n">
         <v>29580</v>
@@ -5906,7 +5906,7 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>29929.47</v>
+        <v>29879.47</v>
       </c>
       <c r="C69" s="2" t="n">
         <v>29450</v>
@@ -5944,7 +5944,7 @@
         </is>
       </c>
       <c r="B70" s="5" t="n">
-        <v>29969.47</v>
+        <v>29919.47</v>
       </c>
       <c r="C70" s="5" t="n">
         <v>29490</v>
@@ -5982,7 +5982,7 @@
         </is>
       </c>
       <c r="B71" s="5" t="n">
-        <v>29779.47</v>
+        <v>29729.47</v>
       </c>
       <c r="C71" s="5" t="n">
         <v>29300</v>
@@ -6016,7 +6016,7 @@
         </is>
       </c>
       <c r="B72" s="5" t="n">
-        <v>30129.47</v>
+        <v>30079.47</v>
       </c>
       <c r="C72" s="5" t="n">
         <v>29650</v>
@@ -6050,7 +6050,7 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>29799.47</v>
+        <v>29749.47</v>
       </c>
       <c r="C73" s="2" t="n">
         <v>29320</v>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>29939.47</v>
+        <v>29889.47</v>
       </c>
       <c r="C74" s="5" t="n">
         <v>29460</v>
@@ -6126,7 +6126,7 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>29829.47</v>
+        <v>29779.47</v>
       </c>
       <c r="C75" s="2" t="n">
         <v>29350</v>
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="B76" s="5" t="n">
-        <v>29854.47</v>
+        <v>29804.47</v>
       </c>
       <c r="C76" s="5" t="n">
         <v>29375</v>
@@ -6202,7 +6202,7 @@
         </is>
       </c>
       <c r="B77" s="5" t="n">
-        <v>29759.47</v>
+        <v>29709.47</v>
       </c>
       <c r="C77" s="5" t="n">
         <v>29280</v>
@@ -6274,7 +6274,7 @@
         </is>
       </c>
       <c r="B79" s="5" t="n">
-        <v>30049.47</v>
+        <v>29999.47</v>
       </c>
       <c r="C79" s="5" t="n">
         <v>29570</v>
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="B80" s="5" t="n">
-        <v>29899.47</v>
+        <v>29849.47</v>
       </c>
       <c r="C80" s="5" t="n">
         <v>29420</v>

</xml_diff>